<commit_message>
docs(dia-chi): dien san 18 tuyen doi ten NQ 380/2025 (theo bang bao Thanh Nien), ghi nguon 52 ap OSM chua chinh thuc
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dia-chi/danh-sach-duong-dong-thanh-nhap.xlsx
+++ b/docs/dia-chi/danh-sach-duong-dong-thanh-nhap.xlsx
@@ -94,7 +94,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">HĐND TP đặt tên 18 tuyến ở Đông Thạnh (NQ 380/NQ-HĐND 24/7/2025). Báo chí mới nêu 2 ví dụ đã điền sẵn; các đường tên đánh số được đánh dấu "Nên kiểm".</t>
+          <t xml:space="preserve">HĐND TP đặt tên 18 tuyến ở Đông Thạnh (NQ 380/NQ-HĐND 24/7/2025). Tên mới đã điền sẵn theo bảng báo Thanh Niên (chưa có bản Công báo) - xã đối chiếu văn bản gốc. "Đông Thạnh 6" bị báo ghi 2 dòng. Tên đánh số khác đánh dấu "Nên kiểm".</t>
         </is>
       </c>
     </row>
@@ -106,7 +106,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Theo ranh giới 52 ấp trên OpenStreetMap. Một đường dài có thể đi qua nhiều ấp. Xã kiểm lại số ấp hiện hành sau sáp nhập.</t>
+          <t xml:space="preserve">Theo ranh giới 52 ấp trên OpenStreetMap (vẽ 9/2026, nguồn là một bài Facebook, chưa phải văn bản). Đợt sắp xếp ấp 6/2026 do HĐND xã quyết. Một đường dài có thể đi qua nhiều ấp. Xã kiểm lại số ấp và ranh giới.</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Trần Thị Hơn</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Đặng Thị Son</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2517,12 +2517,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Thái Thị Mén</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2721,12 +2721,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Huỳnh Thị Xe</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -4285,12 +4285,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phùng Thị Chuyện</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -4965,12 +4965,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nguyễn Thị Nghé</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đt 2-5</t>
+          <t xml:space="preserve">Đê Bao Nhị Bình 22</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -6995,17 +6995,17 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 33, Ấp 39</t>
+          <t xml:space="preserve">Ấp 49</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh</t>
+          <t xml:space="preserve">Nhị Bình</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -7038,7 +7038,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t xml:space="preserve">548993789 607609471</t>
+          <t xml:space="preserve">608247674 608260165</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">ĐT 7</t>
+          <t xml:space="preserve">Đê Bao Sông Sài Gòn</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7063,17 +7063,17 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 44, Ấp 45, Ấp 46</t>
+          <t xml:space="preserve">Ấp 52</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh</t>
+          <t xml:space="preserve">Nhị Bình</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -7098,15 +7098,15 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t xml:space="preserve">residential</t>
+          <t xml:space="preserve">service</t>
         </is>
       </c>
       <c r="M102">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t xml:space="preserve">608194332</t>
+          <t xml:space="preserve">1088092587 1088092589 1448618366 1448618367 1448618371 1448618372 …</t>
         </is>
       </c>
     </row>
@@ -7116,7 +7116,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">ĐT 7-3</t>
+          <t xml:space="preserve">Đông Thạnh 1-3</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 43, Ấp 45, Ấp 46</t>
+          <t xml:space="preserve">Ấp 27, Ấp 28, Ấp 29</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -7174,7 +7174,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889058</t>
+          <t xml:space="preserve">605519832</t>
         </is>
       </c>
     </row>
@@ -7184,7 +7184,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đt 7-4</t>
+          <t xml:space="preserve">Đông Thạnh 1-4</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -7199,7 +7199,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 45, Ấp 46</t>
+          <t xml:space="preserve">Ấp 25, Ấp 27, Ấp 28, Ấp 29</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -7238,11 +7238,11 @@
         </is>
       </c>
       <c r="M104">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889019</t>
+          <t xml:space="preserve">605519833 605519844 605519845</t>
         </is>
       </c>
     </row>
@@ -7252,7 +7252,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đt 7-4A</t>
+          <t xml:space="preserve">Đông Thạnh 1-5</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 46</t>
+          <t xml:space="preserve">Ấp 24</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -7302,15 +7302,15 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t xml:space="preserve">residential, service</t>
+          <t xml:space="preserve">residential</t>
         </is>
       </c>
       <c r="M105">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t xml:space="preserve">1353057048 322889008</t>
+          <t xml:space="preserve">605493787</t>
         </is>
       </c>
     </row>
@@ -7320,7 +7320,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">ĐT 7-5</t>
+          <t xml:space="preserve">Đông Thạnh 2-2</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -7335,7 +7335,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 45</t>
+          <t xml:space="preserve">Ấp 29</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -7378,7 +7378,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t xml:space="preserve">608210317</t>
+          <t xml:space="preserve">607586215</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đê Bao Nhị Bình 22</t>
+          <t xml:space="preserve">Đông Thạnh 2-3</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -7403,17 +7403,17 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 49</t>
+          <t xml:space="preserve">Ấp 24, Ấp 31</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhị Bình</t>
+          <t xml:space="preserve">Đông Thạnh</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -7442,11 +7442,11 @@
         </is>
       </c>
       <c r="M107">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t xml:space="preserve">608247674 608260165</t>
+          <t xml:space="preserve">606247671</t>
         </is>
       </c>
     </row>
@@ -7456,7 +7456,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đê Bao Sông Sài Gòn</t>
+          <t xml:space="preserve">Đông Thạnh 2-3-1</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -7471,17 +7471,17 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 52</t>
+          <t xml:space="preserve">Ấp 24, Ấp 31</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nhị Bình</t>
+          <t xml:space="preserve">Đông Thạnh</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -7506,15 +7506,15 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t xml:space="preserve">service</t>
+          <t xml:space="preserve">residential</t>
         </is>
       </c>
       <c r="M108">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t xml:space="preserve">1088092587 1088092589 1448618366 1448618367 1448618371 1448618372 …</t>
+          <t xml:space="preserve">607577424</t>
         </is>
       </c>
     </row>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 1-3</t>
+          <t xml:space="preserve">Đông Thạnh 2-5</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -7539,7 +7539,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 27, Ấp 28, Ấp 29</t>
+          <t xml:space="preserve">Ấp 33, Ấp 39</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -7549,12 +7549,12 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nguyễn Thị Chồn</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
@@ -7569,7 +7569,7 @@
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Đt 2-5</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7578,11 +7578,11 @@
         </is>
       </c>
       <c r="M109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t xml:space="preserve">605519832</t>
+          <t xml:space="preserve">548993789 607609471</t>
         </is>
       </c>
     </row>
@@ -7592,7 +7592,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 1-4</t>
+          <t xml:space="preserve">Đông Thạnh 2-6</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 25, Ấp 27, Ấp 28, Ấp 29</t>
+          <t xml:space="preserve">Ấp 29, Ấp 30</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ĐT 2-6</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7650,7 +7650,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t xml:space="preserve">605519833 605519844 605519845</t>
+          <t xml:space="preserve">605519827 605519847 607623377</t>
         </is>
       </c>
     </row>
@@ -7660,7 +7660,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 1-5</t>
+          <t xml:space="preserve">Đông Thạnh 2-7</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -7675,7 +7675,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 24</t>
+          <t xml:space="preserve">Ấp 25</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -7718,7 +7718,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t xml:space="preserve">605493787</t>
+          <t xml:space="preserve">605493777</t>
         </is>
       </c>
     </row>
@@ -7728,7 +7728,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 2-2</t>
+          <t xml:space="preserve">Đông Thạnh 3</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 29</t>
+          <t xml:space="preserve">Ấp 28, Ấp 29, Ấp 30, Ấp 33, Ấp 34, Ấp 39</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -7753,12 +7753,12 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nguyễn Thị Út</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -7782,11 +7782,11 @@
         </is>
       </c>
       <c r="M112">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t xml:space="preserve">607586215</t>
+          <t xml:space="preserve">322889021 322889069 531191865 607633457</t>
         </is>
       </c>
     </row>
@@ -7796,7 +7796,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 2-3</t>
+          <t xml:space="preserve">Đông Thạnh 3-1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -7811,7 +7811,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 24, Ấp 31</t>
+          <t xml:space="preserve">Ấp 34, Ấp 39</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t xml:space="preserve">606247671</t>
+          <t xml:space="preserve">531191867</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7864,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 2-3-1</t>
+          <t xml:space="preserve">Đông Thạnh 3-3-1</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -7879,7 +7879,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 24, Ấp 31</t>
+          <t xml:space="preserve">Ấp 29, Ấp 30</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t xml:space="preserve">607577424</t>
+          <t xml:space="preserve">607623378</t>
         </is>
       </c>
     </row>
@@ -7932,7 +7932,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 2-6</t>
+          <t xml:space="preserve">Đông Thạnh 3-4</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -7947,7 +7947,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 29, Ấp 30</t>
+          <t xml:space="preserve">Ấp 30, Ấp 34</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -7977,7 +7977,7 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t xml:space="preserve">ĐT 2-6</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -7986,11 +7986,11 @@
         </is>
       </c>
       <c r="M115">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t xml:space="preserve">605519827 605519847 607623377</t>
+          <t xml:space="preserve">322889111</t>
         </is>
       </c>
     </row>
@@ -8000,7 +8000,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 2-7</t>
+          <t xml:space="preserve">Đông Thạnh 4</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 25</t>
+          <t xml:space="preserve">Ấp 28, Ấp 35, Ấp 36, Ấp 37, Ấp 38, Ấp 39</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -8025,12 +8025,12 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Võ Thị Tới</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t xml:space="preserve">605493777</t>
+          <t xml:space="preserve">322889027</t>
         </is>
       </c>
     </row>
@@ -8068,7 +8068,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 3</t>
+          <t xml:space="preserve">Đông Thạnh 4-1</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 28, Ấp 29, Ấp 30, Ấp 33, Ấp 34, Ấp 39</t>
+          <t xml:space="preserve">Ấp 34, Ấp 35</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -8093,12 +8093,12 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nguyễn Thị Tạo</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
@@ -8122,11 +8122,11 @@
         </is>
       </c>
       <c r="M117">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889021 322889069 531191865 607633457</t>
+          <t xml:space="preserve">607623347 607623348</t>
         </is>
       </c>
     </row>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 3-1</t>
+          <t xml:space="preserve">Đông Thạnh 4-2</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -8151,7 +8151,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 34, Ấp 39</t>
+          <t xml:space="preserve">Ấp 28, Ấp 34, Ấp 35</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -8194,7 +8194,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t xml:space="preserve">531191867</t>
+          <t xml:space="preserve">322889046</t>
         </is>
       </c>
     </row>
@@ -8204,7 +8204,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 3-3-1</t>
+          <t xml:space="preserve">Đông Thạnh 4-2 Nhánh 1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -8219,7 +8219,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 29, Ấp 30</t>
+          <t xml:space="preserve">Ấp 28, Ấp 30, Ấp 34</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t xml:space="preserve">607623378</t>
+          <t xml:space="preserve">322889116</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8272,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 3-4</t>
+          <t xml:space="preserve">Đông Thạnh 5</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -8287,7 +8287,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 30, Ấp 34</t>
+          <t xml:space="preserve">Ấp 35, Ấp 37, Ấp 38</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -8297,12 +8297,12 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nguyễn Thị Tạo</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
@@ -8326,11 +8326,11 @@
         </is>
       </c>
       <c r="M120">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889111</t>
+          <t xml:space="preserve">322889109 608176953</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 4</t>
+          <t xml:space="preserve">Đông Thạnh 6</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 28, Ấp 35, Ấp 36, Ấp 37, Ấp 38, Ấp 39</t>
+          <t xml:space="preserve">Ấp 35, Ấp 37, Ấp 38, Ấp 42, Ấp 43</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -8365,12 +8365,12 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Trương Thị Trưng hoặc Nguyễn Thị Dễ (báo ghi 2 dòng, cần văn bản gốc)</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
@@ -8394,11 +8394,11 @@
         </is>
       </c>
       <c r="M121">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889027</t>
+          <t xml:space="preserve">322889009 322889013 322889029 322889118</t>
         </is>
       </c>
     </row>
@@ -8408,7 +8408,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 4-1</t>
+          <t xml:space="preserve">Đông Thạnh 6-4</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 34, Ấp 35</t>
+          <t xml:space="preserve">Ấp 43</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -8453,12 +8453,12 @@
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Đt 6-4</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t xml:space="preserve">residential</t>
+          <t xml:space="preserve">residential, service</t>
         </is>
       </c>
       <c r="M122">
@@ -8466,7 +8466,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t xml:space="preserve">607623347 607623348</t>
+          <t xml:space="preserve">1181704181 608194340</t>
         </is>
       </c>
     </row>
@@ -8476,7 +8476,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 4-2</t>
+          <t xml:space="preserve">Đông Thạnh 7</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -8491,7 +8491,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 28, Ấp 34, Ấp 35</t>
+          <t xml:space="preserve">Ấp 44, Ấp 45, Ấp 46</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -8501,12 +8501,12 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lê Thị Thìn</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ĐT 7</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -8534,7 +8534,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889046</t>
+          <t xml:space="preserve">608194332</t>
         </is>
       </c>
     </row>
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 4-2 Nhánh 1</t>
+          <t xml:space="preserve">Đông Thạnh 7-1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 28, Ấp 30, Ấp 34</t>
+          <t xml:space="preserve">Ấp 40, Ấp 47</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889116</t>
+          <t xml:space="preserve">322889011</t>
         </is>
       </c>
     </row>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 5</t>
+          <t xml:space="preserve">Đông Thạnh 7-1-1</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -8627,7 +8627,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 35, Ấp 37, Ấp 38</t>
+          <t xml:space="preserve">Ấp 47</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889109 608176953</t>
+          <t xml:space="preserve">322889110 608198800</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 6</t>
+          <t xml:space="preserve">Đông Thạnh 7-2</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 35, Ấp 37, Ấp 38, Ấp 42, Ấp 43</t>
+          <t xml:space="preserve">Ấp 47</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -8705,12 +8705,12 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có (báo chí)</t>
+          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trương Thị Trưng</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -8734,11 +8734,11 @@
         </is>
       </c>
       <c r="M126">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889009 322889013 322889029 322889118</t>
+          <t xml:space="preserve">322889112</t>
         </is>
       </c>
     </row>
@@ -8748,7 +8748,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 6-4</t>
+          <t xml:space="preserve">Đông Thạnh 7-3</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -8763,7 +8763,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 43</t>
+          <t xml:space="preserve">Ấp 43, Ấp 45, Ấp 46</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -8773,12 +8773,12 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phạm Thị Tôm</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -8793,20 +8793,20 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đt 6-4</t>
+          <t xml:space="preserve">ĐT 7-3</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t xml:space="preserve">residential, service</t>
+          <t xml:space="preserve">residential</t>
         </is>
       </c>
       <c r="M127">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t xml:space="preserve">1181704181 608194340</t>
+          <t xml:space="preserve">322889058</t>
         </is>
       </c>
     </row>
@@ -8816,7 +8816,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 7-1</t>
+          <t xml:space="preserve">Đông Thạnh 7-4</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -8831,7 +8831,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 40, Ấp 47</t>
+          <t xml:space="preserve">Ấp 45, Ấp 46</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -8841,12 +8841,12 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nên kiểm (tên đánh số)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nguyễn Thị Đẹt</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
@@ -8861,7 +8861,7 @@
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Đt 7-4</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889011</t>
+          <t xml:space="preserve">322889019</t>
         </is>
       </c>
     </row>
@@ -8884,7 +8884,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 7-1-1</t>
+          <t xml:space="preserve">Đông Thạnh 7-4A</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -8899,7 +8899,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 47</t>
+          <t xml:space="preserve">Ấp 46</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -8929,12 +8929,12 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Đt 7-4A</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t xml:space="preserve">residential</t>
+          <t xml:space="preserve">residential, service</t>
         </is>
       </c>
       <c r="M129">
@@ -8942,7 +8942,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889110 608198800</t>
+          <t xml:space="preserve">1353057048 322889008</t>
         </is>
       </c>
     </row>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đông Thạnh 7-2</t>
+          <t xml:space="preserve">Đông Thạnh 7-5</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ấp 47</t>
+          <t xml:space="preserve">Ấp 45</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ĐT 7-5</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -9010,7 +9010,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t xml:space="preserve">322889112</t>
+          <t xml:space="preserve">608210317</t>
         </is>
       </c>
     </row>
@@ -9045,7 +9045,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Có (báo chí)</t>
+          <t xml:space="preserve">Có (NQ 380, theo báo)</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -12970,7 +12970,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huỳnh Thị Na; Đt 2-5; Đông Thạnh 3; Đặng Thúc Vịnh</t>
+          <t xml:space="preserve">Huỳnh Thị Na; Đông Thạnh 2-5; Đông Thạnh 3; Đặng Thúc Vịnh</t>
         </is>
       </c>
     </row>
@@ -13090,7 +13090,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lê Văn Khương; Nhánh 1; Trần Văn Danh; Trịnh Thị Dối; Đt 2-5; Đông Thạnh 3; Đông Thạnh 3-1; Đông Thạnh 4; Đặng Thúc Vịnh</t>
+          <t xml:space="preserve">Lê Văn Khương; Nhánh 1; Trần Văn Danh; Trịnh Thị Dối; Đông Thạnh 2-5; Đông Thạnh 3; Đông Thạnh 3-1; Đông Thạnh 4; Đặng Thúc Vịnh</t>
         </is>
       </c>
     </row>
@@ -13170,7 +13170,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lê Văn Khương; Nguyễn Thị Dễ; Trịnh Thị Dối; ĐT 7-3; Đông Thạnh 6; Đông Thạnh 6-4</t>
+          <t xml:space="preserve">Lê Văn Khương; Nguyễn Thị Dễ; Trịnh Thị Dối; Đông Thạnh 6; Đông Thạnh 6-4; Đông Thạnh 7-3</t>
         </is>
       </c>
     </row>
@@ -13190,7 +13190,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Dừa; Hẻm 98/50; Lê Văn Khương; Trịnh Thị Dối; ĐT 7; Đông Thạnh 8</t>
+          <t xml:space="preserve">Cầu Dừa; Hẻm 98/50; Lê Văn Khương; Trịnh Thị Dối; Đông Thạnh 7; Đông Thạnh 8</t>
         </is>
       </c>
     </row>
@@ -13210,7 +13210,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cầu Bến Đá; Hẻm 98/50; Trịnh Thị Dối; ĐT 7; ĐT 7-3; Đt 7-4; ĐT 7-5; Đông Thạnh 8</t>
+          <t xml:space="preserve">Cầu Bến Đá; Hẻm 98/50; Trịnh Thị Dối; Đông Thạnh 7; Đông Thạnh 7-3; Đông Thạnh 7-4; Đông Thạnh 7-5; Đông Thạnh 8</t>
         </is>
       </c>
     </row>
@@ -13230,7 +13230,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bùi Công Trừng; Cầu Bến Đá; Trịnh Thị Dối; ĐT 7; ĐT 7-3; Đt 7-4; Đt 7-4A</t>
+          <t xml:space="preserve">Bùi Công Trừng; Cầu Bến Đá; Trịnh Thị Dối; Đông Thạnh 7; Đông Thạnh 7-3; Đông Thạnh 7-4; Đông Thạnh 7-4A</t>
         </is>
       </c>
     </row>

</xml_diff>